<commit_message>
Next update part 3: my profile (the center node)
- New Me sheet (Field | Value): name, photo, role, headline, company,
  schools, past companies, email, LinkedIn, location, what I'm looking
  for; a name typed there wins; setProfile edit
- Clicking the center node (or Settings > Edit my profile) opens your
  profile in the sidebar, every field click-to-edit, Change photo
- Your photo on the center node; 'Same school' and 'Former coworker'
  badges on people's details and chip lists on your profile, matched
  through org aliases
- Demo: Alex Rivera gets an AI-generated SFHQ headshot (source listed)
  and a full fictional student profile

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -9,9 +9,10 @@
     <sheet name="LinkedIn Pool" sheetId="4" r:id="rId4"/>
     <sheet name="Meetings" sheetId="5" r:id="rId5"/>
     <sheet name="Tasks" sheetId="6" r:id="rId6"/>
-    <sheet name="Settings" sheetId="7" r:id="rId7"/>
-    <sheet name="Layout" sheetId="8" r:id="rId8" state="hidden"/>
-    <sheet name="How to use" sheetId="9" r:id="rId9"/>
+    <sheet name="Me" sheetId="7" r:id="rId7"/>
+    <sheet name="Settings" sheetId="8" r:id="rId8"/>
+    <sheet name="Layout" sheetId="9" r:id="rId9" state="hidden"/>
+    <sheet name="How to use" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -1374,6 +1375,173 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B19"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="110.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Sheet / column</v>
+      </c>
+      <c r="B1" t="str">
+        <v>What to put there</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>People</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Everyone on your map. Only Name is required.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v xml:space="preserve">  Name</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Full name, spelled the same way everywhere.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v xml:space="preserve">  Company / School</v>
+      </c>
+      <c r="B4" t="str">
+        <v>3+ direct connections at one company or school become a group bubble. 'Stanford' and 'Stanford University' count as the same.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v xml:space="preserve">  Email</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Shown in the details panel with a copy button.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v xml:space="preserve">  LinkedIn URL</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Their profile link. Double-click them on the map to open it.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v xml:space="preserve">  Photo</v>
+      </c>
+      <c r="B7" t="str">
+        <v>An image link, or use 'Add photo' in the app (it stores a small picture here). LinkedIn exports don't include photos.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">  Connected Through</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Leave BLANK if you know them directly. Otherwise put the name of the person who connects you; they appear as a 2nd-degree connection.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v xml:space="preserve">  Connected On</v>
+      </c>
+      <c r="B9" t="str">
+        <v>The date you connected (filled in from LinkedIn).</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v xml:space="preserve">  Status</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Met / Contacted / To Reach Out / Follow Up / Referral.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">  Tags, Notes</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Anything you want to remember. Tags are comma-separated.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Targets</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Companies you want to work at. Priority (1 = highest) and Stage (Researching / Networking / Applied / Interviewing / Offer) are optional.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Companies</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Optional. Set a company's Website (e.g. byu.edu) if its logo comes out wrong, or put an image link in Logo.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>LinkedIn Pool</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Filled by 'Import LinkedIn' from your Connections.csv. These people are NOT on the map until you add them.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Meetings</v>
+      </c>
+      <c r="B15" t="str">
+        <v>One row per meeting: Person, Date, Start, End, Type, Method, Notes, Next Step. The app fills this when you schedule or log a meeting.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Tasks</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Your to-dos: Task, Person, Company, Due, Done. Scheduling a meeting adds a 'Send thank-you' task automatically.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Settings</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Your name and email, default meeting length, your Zoom link (used in invites), the invite message, and Avatar style (initials or notionists).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Layout</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Managed by the app (saved node positions).</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Privacy</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Network Map runs entirely in your browser. This file is never uploaded anywhere.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D7"/>
@@ -2935,6 +3103,118 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" customWidth="1" width="22.83203125"/>
+    <col min="2" max="2" customWidth="1" width="70.83203125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Alex Rivera</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Photo</v>
+      </c>
+      <c r="B3" t="str">
+        <v>demo/photos/alex-rivera.jpg</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Role</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MBA Candidate</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Headline</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Stanford MBA '27 · Looking for strategy &amp; product roles</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Company</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Schools</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Stanford University (2025–2027); University of Utah (2016–2020)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Past Companies</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Delta Air Lines (2020–2022); Adobe (2022–2025)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Email</v>
+      </c>
+      <c r="B9" t="str">
+        <v>alex.rivera@example.com</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>LinkedIn URL</v>
+      </c>
+      <c r="B10" t="str">
+        <v>https://www.linkedin.com/in/alex-rivera-demo</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Location</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Palo Alto, California</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>What I'm looking for</v>
+      </c>
+      <c r="B12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Summer 2027 internships in strategy or product at consumer-tech and airline companies.
+Happy to swap notes on case prep and product sense interviews.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="26.83203125"/>
@@ -3020,7 +3300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C1"/>
   <cols>
@@ -3045,171 +3325,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="110.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Sheet / column</v>
-      </c>
-      <c r="B1" t="str">
-        <v>What to put there</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>People</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Everyone on your map. Only Name is required.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v xml:space="preserve">  Name</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Full name, spelled the same way everywhere.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v xml:space="preserve">  Company / School</v>
-      </c>
-      <c r="B4" t="str">
-        <v>3+ direct connections at one company or school become a group bubble. 'Stanford' and 'Stanford University' count as the same.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v xml:space="preserve">  Email</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Shown in the details panel with a copy button.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v xml:space="preserve">  LinkedIn URL</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Their profile link. Double-click them on the map to open it.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v xml:space="preserve">  Photo</v>
-      </c>
-      <c r="B7" t="str">
-        <v>An image link, or use 'Add photo' in the app (it stores a small picture here). LinkedIn exports don't include photos.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v xml:space="preserve">  Connected Through</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Leave BLANK if you know them directly. Otherwise put the name of the person who connects you; they appear as a 2nd-degree connection.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v xml:space="preserve">  Connected On</v>
-      </c>
-      <c r="B9" t="str">
-        <v>The date you connected (filled in from LinkedIn).</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v xml:space="preserve">  Status</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Met / Contacted / To Reach Out / Follow Up / Referral.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v xml:space="preserve">  Tags, Notes</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Anything you want to remember. Tags are comma-separated.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Targets</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Companies you want to work at. Priority (1 = highest) and Stage (Researching / Networking / Applied / Interviewing / Offer) are optional.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Companies</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Optional. Set a company's Website (e.g. byu.edu) if its logo comes out wrong, or put an image link in Logo.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>LinkedIn Pool</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Filled by 'Import LinkedIn' from your Connections.csv. These people are NOT on the map until you add them.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Meetings</v>
-      </c>
-      <c r="B15" t="str">
-        <v>One row per meeting: Person, Date, Start, End, Type, Method, Notes, Next Step. The app fills this when you schedule or log a meeting.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Tasks</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Your to-dos: Task, Person, Company, Due, Done. Scheduling a meeting adds a 'Send thank-you' task automatically.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Settings</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Your name and email, default meeting length, your Zoom link (used in invites), the invite message, and Avatar style (initials or notionists).</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Layout</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Managed by the app (saved node positions).</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Privacy</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Network Map runs entirely in your browser. This file is never uploaded anywhere.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Next update part 4: connections between people
- Connections sheet (Person A, Person B, Type, Notes); types: Introduced
  me, Coworker, Classmate, Friend, Mentor, Other (free text). The old
  Connected Through column migrates in and stays in People, kept in sync
  from 'Introduced me' (edits typed there in Excel still import)
- Only 'Introduced me' makes someone 2nd-degree; other types draw purple
  person-to-person links (in highlight-on-click, legend)
- Best path is now a breadth-first search from you over introductions
  and person links (warmest first contact wins ties; alumni fallback)
- Connections section in person details (add with type-ahead + type,
  remove from either side) and in the Add-person review card (several
  rows); renames and removals carry through
- Demo: four links (friend, classmate, mentor, coworker)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -9,10 +9,11 @@
     <sheet name="LinkedIn Pool" sheetId="4" r:id="rId4"/>
     <sheet name="Meetings" sheetId="5" r:id="rId5"/>
     <sheet name="Tasks" sheetId="6" r:id="rId6"/>
-    <sheet name="Me" sheetId="7" r:id="rId7"/>
-    <sheet name="Settings" sheetId="8" r:id="rId8"/>
-    <sheet name="Layout" sheetId="9" r:id="rId9" state="hidden"/>
-    <sheet name="How to use" sheetId="10" r:id="rId10"/>
+    <sheet name="Connections" sheetId="7" r:id="rId7"/>
+    <sheet name="Me" sheetId="8" r:id="rId8"/>
+    <sheet name="Settings" sheetId="9" r:id="rId9"/>
+    <sheet name="Layout" sheetId="10" r:id="rId10" state="hidden"/>
+    <sheet name="How to use" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -1377,7 +1378,34 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" customWidth="1" width="36.83203125"/>
+    <col min="2" max="2" customWidth="1" width="8.83203125"/>
+    <col min="3" max="3" customWidth="1" width="8.83203125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Node</v>
+      </c>
+      <c r="B1" t="str">
+        <v>X</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B21"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -1497,47 +1525,63 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Meetings</v>
+        <v>Connections</v>
       </c>
       <c r="B15" t="str">
-        <v>One row per meeting: Person, Date, Start, End, Type, Method, Notes, Next Step. The app fills this when you schedule or log a meeting.</v>
+        <v>Who knows whom: Person A, Person B, Type (Introduced me, Coworker, Classmate, Friend, Mentor, or anything else), Notes. 'Introduced me' means A introduced you to B; it's kept in sync with People → Connected Through.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Tasks</v>
+        <v>Me</v>
       </c>
       <c r="B16" t="str">
-        <v>Your to-dos: Task, Person, Company, Due, Done. Scheduling a meeting adds a 'Send thank-you' task automatically.</v>
+        <v>Your own profile: photo, role, schools, past companies, what you're looking for.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Settings</v>
+        <v>Meetings</v>
       </c>
       <c r="B17" t="str">
-        <v>Your name and email, default meeting length, your Zoom link (used in invites), the invite message, and Avatar style (initials or notionists).</v>
+        <v>One row per meeting: Person, Date, Start, End, Type, Method, Notes, Next Step. The app fills this when you schedule or log a meeting.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Layout</v>
+        <v>Tasks</v>
       </c>
       <c r="B18" t="str">
-        <v>Managed by the app (saved node positions).</v>
+        <v>Your to-dos: Task, Person, Company, Due, Done. Scheduling a meeting adds a 'Send thank-you' task automatically.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>Settings</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Your name and email, default meeting length, your Zoom link (used in invites), the invite message, and Avatar style (initials or notionists).</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Layout</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Managed by the app (saved node positions).</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
         <v>Privacy</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B21" t="str">
         <v>Network Map runs entirely in your browser. This file is never uploaded anywhere.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3103,6 +3147,205 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D13"/>
+  <cols>
+    <col min="1" max="1" customWidth="1" width="24.83203125"/>
+    <col min="2" max="2" customWidth="1" width="24.83203125"/>
+    <col min="3" max="3" customWidth="1" width="16.83203125"/>
+    <col min="4" max="4" customWidth="1" width="40.83203125"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Person A</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Person B</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Rachel Green</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Tom Nguyen</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Isla Moore</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Noah Carter</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Victor Hale</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Mia Chen</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Chloe Park</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Daniel Ortiz</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Ben Foster</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Liam Walsh</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Zoe Adams</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Zoe Adams</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Sam Rivera</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Introduced me</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Liam Walsh</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Mia Chen</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Friend</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Roommates' friend group</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Daniel Ortiz</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Classmate</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Stanford, same product club</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Owen Price</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Mentor</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Jordan mentors Owen on case interviews</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Hana Kim</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Ethan Brooks</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Coworker</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Worked together at Deloitte</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="22.83203125"/>
@@ -3213,7 +3456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B9"/>
   <cols>
@@ -3298,31 +3541,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
-  <cols>
-    <col min="1" max="1" customWidth="1" width="36.83203125"/>
-    <col min="2" max="2" customWidth="1" width="8.83203125"/>
-    <col min="3" max="3" customWidth="1" width="8.83203125"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Node</v>
-      </c>
-      <c r="B1" t="str">
-        <v>X</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixes part 3: easy Excel export
An Export button in the top bar (every view) and Cmd/Ctrl+E: Everything, This
view (highlighted people on the map, the filtered LinkedIn pool, open tasks, or
the calendar's meetings), or One person (also from their details). People come
out in the networking-tracker layout with derived columns (How We're Connected,
meeting, follow-up, next steps) filled in and LinkedIn as a Profile link.

Every workbook Orbit writes now has a frozen bold header, auto column widths,
wrapped long text, clickable links and dropdowns (added to the xlsx XML with
the zip reader inside SheetJS). Exports open in Orbit again with the same data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -4,17 +4,23 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="People" sheetId="1" r:id="rId1"/>
-    <sheet name="Targets" sheetId="2" r:id="rId2"/>
-    <sheet name="Companies" sheetId="3" r:id="rId3"/>
-    <sheet name="LinkedIn Pool" sheetId="4" r:id="rId4"/>
-    <sheet name="Meetings" sheetId="5" r:id="rId5"/>
-    <sheet name="Tasks" sheetId="6" r:id="rId6"/>
-    <sheet name="Connections" sheetId="7" r:id="rId7"/>
-    <sheet name="Me" sheetId="8" r:id="rId8"/>
-    <sheet name="Settings" sheetId="9" r:id="rId9"/>
-    <sheet name="Layout" sheetId="10" r:id="rId10" state="hidden"/>
-    <sheet name="How to use" sheetId="11" r:id="rId11"/>
+    <sheet name="How to use" sheetId="2" r:id="rId2"/>
+    <sheet name="Targets" sheetId="3" r:id="rId3"/>
+    <sheet name="Companies" sheetId="4" r:id="rId4"/>
+    <sheet name="LinkedIn Pool" sheetId="5" r:id="rId5"/>
+    <sheet name="Meetings" sheetId="6" r:id="rId6"/>
+    <sheet name="Tasks" sheetId="7" r:id="rId7"/>
+    <sheet name="Connections" sheetId="8" r:id="rId8"/>
+    <sheet name="Experience" sheetId="9" r:id="rId9"/>
+    <sheet name="Education" sheetId="10" r:id="rId10"/>
+    <sheet name="Me" sheetId="11" r:id="rId11"/>
+    <sheet name="Settings" sheetId="12" r:id="rId12"/>
+    <sheet name="Layout" sheetId="13" r:id="rId13" state="hidden"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">People!$A$1:$U$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'LinkedIn Pool'!$A$1:$G$27</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -46,8 +52,16 @@
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
     <numFmt numFmtId="60" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -75,9 +89,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,62 +429,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:U23"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="22.83203125"/>
-    <col min="2" max="2" customWidth="1" width="24.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="24.83203125"/>
-    <col min="5" max="5" customWidth="1" width="28.83203125"/>
-    <col min="6" max="6" customWidth="1" width="36.83203125"/>
-    <col min="7" max="7" customWidth="1" width="14.83203125"/>
-    <col min="8" max="8" customWidth="1" width="22.83203125"/>
-    <col min="9" max="9" customWidth="1" width="14.83203125"/>
-    <col min="10" max="10" customWidth="1" width="14.83203125"/>
-    <col min="11" max="11" customWidth="1" width="20.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125"/>
-    <col min="13" max="13" customWidth="1" width="36.83203125"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="5" max="5" width="27.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="31.83203125" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" customWidth="1"/>
+    <col min="16" max="16" width="9.83203125" customWidth="1"/>
+    <col min="17" max="17" width="8.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1"/>
+    <col min="19" max="19" width="16.83203125" customWidth="1"/>
+    <col min="20" max="20" width="8.83203125" customWidth="1"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Schools</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>Role</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" t="str" s="2">
         <v>Email</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" t="str" s="2">
         <v>LinkedIn URL</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" t="str" s="2">
         <v>Photo</v>
       </c>
-      <c r="H1" t="str">
+      <c r="H1" t="str" s="2">
         <v>Connected Through</v>
       </c>
-      <c r="I1" t="str">
+      <c r="I1" t="str" s="2">
         <v>Connected On</v>
       </c>
-      <c r="J1" t="str">
+      <c r="J1" t="str" s="2">
         <v>Status</v>
       </c>
-      <c r="K1" t="str">
+      <c r="K1" t="str" s="2">
         <v>Tags</v>
       </c>
-      <c r="L1" t="str">
+      <c r="L1" t="str" s="2">
         <v>Notes</v>
       </c>
-      <c r="M1" t="str">
+      <c r="M1" t="str" s="2">
         <v>Past Companies</v>
+      </c>
+      <c r="N1" t="str" s="2">
+        <v>Headline</v>
+      </c>
+      <c r="O1" t="str" s="2">
+        <v>Location</v>
+      </c>
+      <c r="P1" t="str" s="2">
+        <v>Website</v>
+      </c>
+      <c r="Q1" t="str" s="2">
+        <v>Skills</v>
+      </c>
+      <c r="R1" t="str" s="2">
+        <v>Languages</v>
+      </c>
+      <c r="S1" t="str" s="2">
+        <v>Certifications</v>
+      </c>
+      <c r="T1" t="str" s="2">
+        <v>Honors</v>
+      </c>
+      <c r="U1" t="str" s="2">
+        <v>About</v>
       </c>
     </row>
     <row r="2">
@@ -474,7 +526,7 @@
       <c r="B2" t="str">
         <v>Deloitte</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C2" t="str" s="3">
         <v>Stanford University</v>
       </c>
       <c r="D2" t="str">
@@ -501,10 +553,34 @@
       <c r="K2" t="str">
         <v>Consulting club</v>
       </c>
-      <c r="L2" t="str">
+      <c r="L2" t="str" s="3">
         <v>Case interview tips</v>
       </c>
-      <c r="M2" t="str">
+      <c r="M2" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N2" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -515,7 +591,7 @@
       <c r="B3" t="str">
         <v>Deloitte</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C3" t="str" s="3">
         <v>University of Utah</v>
       </c>
       <c r="D3" t="str">
@@ -542,10 +618,34 @@
       <c r="K3" t="str">
         <v/>
       </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+      <c r="L3" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M3" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N3" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -556,7 +656,7 @@
       <c r="B4" t="str">
         <v>Microsoft</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" t="str" s="3">
         <v>Stanford University</v>
       </c>
       <c r="D4" t="str">
@@ -583,10 +683,34 @@
       <c r="K4" t="str">
         <v>Product</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L4" t="str" s="3">
         <v>Owns the marketplace roadmap</v>
       </c>
-      <c r="M4" t="str">
+      <c r="M4" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N4" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -597,7 +721,7 @@
       <c r="B5" t="str">
         <v>Delta Air Lines</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" t="str" s="3">
         <v>Stanford University</v>
       </c>
       <c r="D5" t="str">
@@ -624,10 +748,34 @@
       <c r="K5" t="str">
         <v/>
       </c>
-      <c r="L5" t="str">
+      <c r="L5" t="str" s="3">
         <v>Info session speaker</v>
       </c>
-      <c r="M5" t="str">
+      <c r="M5" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N5" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -638,7 +786,7 @@
       <c r="B6" t="str">
         <v>Google</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6" t="str" s="3">
         <v>University of Utah</v>
       </c>
       <c r="D6" t="str">
@@ -665,10 +813,34 @@
       <c r="K6" t="str">
         <v/>
       </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
+      <c r="L6" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M6" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N6" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -679,7 +851,7 @@
       <c r="B7" t="str">
         <v>Deloitte</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7" t="str" s="3">
         <v>Stanford</v>
       </c>
       <c r="D7" t="str">
@@ -706,10 +878,34 @@
       <c r="K7" t="str">
         <v>Consulting club</v>
       </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
+      <c r="L7" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M7" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N7" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -720,7 +916,7 @@
       <c r="B8" t="str">
         <v>Deloitte LLP</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C8" t="str" s="3">
         <v/>
       </c>
       <c r="D8" t="str">
@@ -747,10 +943,34 @@
       <c r="K8" t="str">
         <v/>
       </c>
-      <c r="L8" t="str">
+      <c r="L8" t="str" s="3">
         <v>Leads the strategy practice</v>
       </c>
-      <c r="M8" t="str">
+      <c r="M8" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N8" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -761,7 +981,7 @@
       <c r="B9" t="str">
         <v>Microsoft</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C9" t="str" s="3">
         <v/>
       </c>
       <c r="D9" t="str">
@@ -788,10 +1008,34 @@
       <c r="K9" t="str">
         <v>Product</v>
       </c>
-      <c r="L9" t="str">
-        <v/>
-      </c>
-      <c r="M9" t="str">
+      <c r="L9" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M9" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N9" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -802,7 +1046,7 @@
       <c r="B10" t="str">
         <v>Microsoft</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C10" t="str" s="3">
         <v>University of Utah</v>
       </c>
       <c r="D10" t="str">
@@ -829,10 +1073,34 @@
       <c r="K10" t="str">
         <v>Product</v>
       </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10" t="str">
+      <c r="L10" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M10" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N10" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -843,7 +1111,7 @@
       <c r="B11" t="str">
         <v>Delta Air Lines</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C11" t="str" s="3">
         <v/>
       </c>
       <c r="D11" t="str">
@@ -870,10 +1138,34 @@
       <c r="K11" t="str">
         <v/>
       </c>
-      <c r="L11" t="str">
-        <v/>
-      </c>
-      <c r="M11" t="str">
+      <c r="L11" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M11" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N11" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -884,7 +1176,7 @@
       <c r="B12" t="str">
         <v>Goldman Sachs</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" t="str" s="3">
         <v>Stanford University</v>
       </c>
       <c r="D12" t="str">
@@ -911,10 +1203,34 @@
       <c r="K12" t="str">
         <v/>
       </c>
-      <c r="L12" t="str">
-        <v/>
-      </c>
-      <c r="M12" t="str">
+      <c r="L12" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M12" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N12" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -925,7 +1241,7 @@
       <c r="B13" t="str">
         <v>Google</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" t="str" s="3">
         <v>University of Utah</v>
       </c>
       <c r="D13" t="str">
@@ -952,10 +1268,34 @@
       <c r="K13" t="str">
         <v/>
       </c>
-      <c r="L13" t="str">
-        <v/>
-      </c>
-      <c r="M13" t="str">
+      <c r="L13" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M13" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N13" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -966,7 +1306,7 @@
       <c r="B14" t="str">
         <v>Adobe</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" t="str" s="3">
         <v>University of Utah</v>
       </c>
       <c r="D14" t="str">
@@ -993,10 +1333,34 @@
       <c r="K14" t="str">
         <v/>
       </c>
-      <c r="L14" t="str">
-        <v/>
-      </c>
-      <c r="M14" t="str">
+      <c r="L14" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M14" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N14" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1007,7 +1371,7 @@
       <c r="B15" t="str">
         <v>Independent</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" t="str" s="3">
         <v/>
       </c>
       <c r="D15" t="str">
@@ -1034,10 +1398,34 @@
       <c r="K15" t="str">
         <v/>
       </c>
-      <c r="L15" t="str">
+      <c r="L15" t="str" s="3">
         <v>Old roommate</v>
       </c>
-      <c r="M15" t="str">
+      <c r="M15" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N15" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1048,7 +1436,7 @@
       <c r="B16" t="str">
         <v>Deloitte</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" t="str" s="3">
         <v/>
       </c>
       <c r="D16" t="str">
@@ -1075,10 +1463,34 @@
       <c r="K16" t="str">
         <v/>
       </c>
-      <c r="L16" t="str">
+      <c r="L16" t="str" s="3">
         <v>Jordan offered an intro</v>
       </c>
-      <c r="M16" t="str">
+      <c r="M16" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N16" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1089,7 +1501,7 @@
       <c r="B17" t="str">
         <v>Microsoft</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C17" t="str" s="3">
         <v/>
       </c>
       <c r="D17" t="str">
@@ -1116,10 +1528,34 @@
       <c r="K17" t="str">
         <v>Product</v>
       </c>
-      <c r="L17" t="str">
-        <v/>
-      </c>
-      <c r="M17" t="str">
+      <c r="L17" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M17" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N17" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1130,7 +1566,7 @@
       <c r="B18" t="str">
         <v>Microsoft</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C18" t="str" s="3">
         <v/>
       </c>
       <c r="D18" t="str">
@@ -1157,10 +1593,34 @@
       <c r="K18" t="str">
         <v>Product</v>
       </c>
-      <c r="L18" t="str">
-        <v/>
-      </c>
-      <c r="M18" t="str">
+      <c r="L18" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M18" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N18" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1171,7 +1631,7 @@
       <c r="B19" t="str">
         <v>Delta Air Lines</v>
       </c>
-      <c r="C19" t="str">
+      <c r="C19" t="str" s="3">
         <v/>
       </c>
       <c r="D19" t="str">
@@ -1198,10 +1658,34 @@
       <c r="K19" t="str">
         <v/>
       </c>
-      <c r="L19" t="str">
-        <v/>
-      </c>
-      <c r="M19" t="str">
+      <c r="L19" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M19" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N19" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1212,7 +1696,7 @@
       <c r="B20" t="str">
         <v>Adobe</v>
       </c>
-      <c r="C20" t="str">
+      <c r="C20" t="str" s="3">
         <v/>
       </c>
       <c r="D20" t="str">
@@ -1239,10 +1723,34 @@
       <c r="K20" t="str">
         <v/>
       </c>
-      <c r="L20" t="str">
-        <v/>
-      </c>
-      <c r="M20" t="str">
+      <c r="L20" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M20" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N20" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1253,7 +1761,7 @@
       <c r="B21" t="str">
         <v>Stanford University</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C21" t="str" s="3">
         <v/>
       </c>
       <c r="D21" t="str">
@@ -1280,10 +1788,34 @@
       <c r="K21" t="str">
         <v/>
       </c>
-      <c r="L21" t="str">
-        <v/>
-      </c>
-      <c r="M21" t="str">
+      <c r="L21" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M21" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N21" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1294,7 +1826,7 @@
       <c r="B22" t="str">
         <v>Qualtrics</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C22" t="str" s="3">
         <v/>
       </c>
       <c r="D22" t="str">
@@ -1321,10 +1853,34 @@
       <c r="K22" t="str">
         <v/>
       </c>
-      <c r="L22" t="str">
-        <v/>
-      </c>
-      <c r="M22" t="str">
+      <c r="L22" t="str" s="3">
+        <v/>
+      </c>
+      <c r="M22" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N22" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1335,7 +1891,7 @@
       <c r="B23" t="str">
         <v>Qualtrics</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C23" t="str" s="3">
         <v/>
       </c>
       <c r="D23" t="str">
@@ -1362,27 +1918,311 @@
       <c r="K23" t="str">
         <v/>
       </c>
-      <c r="L23" t="str">
+      <c r="L23" t="str" s="3">
         <v>3rd-degree example</v>
       </c>
-      <c r="M23" t="str">
+      <c r="M23" t="str" s="3">
+        <v/>
+      </c>
+      <c r="N23" t="str" s="3">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str" s="3">
         <v/>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U23"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="J2:J1000">
+      <formula1>"To Reach Out,Contacted,Scheduled,Met,Follow Up,Referral"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" display="jordan.lee@example.com"/>
+    <hyperlink ref="E3" r:id="rId2" display="priya.shah@example.com"/>
+    <hyperlink ref="E4" r:id="rId3" display="sofia.alvarez@example.com"/>
+    <hyperlink ref="E5" r:id="rId4" display="noah.carter@example.com"/>
+    <hyperlink ref="E6" r:id="rId5" display="mia.chen@example.com"/>
+    <hyperlink ref="E7" r:id="rId6" display="marcus.bell@example.com"/>
+    <hyperlink ref="E8" r:id="rId7" display="hana.kim@example.com"/>
+    <hyperlink ref="E9" r:id="rId8" display="ethan.brooks@example.com"/>
+    <hyperlink ref="E10" r:id="rId9" display="lena.novak@example.com"/>
+    <hyperlink ref="E11" r:id="rId10" display="grace.owens@example.com"/>
+    <hyperlink ref="E12" r:id="rId11" display="daniel.ortiz@example.com"/>
+    <hyperlink ref="E13" r:id="rId12" display="owen.price@example.com"/>
+    <hyperlink ref="E14" r:id="rId13" display="ava.thompson@example.com"/>
+    <hyperlink ref="E15" r:id="rId14" display="liam.walsh@example.com"/>
+  </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str" s="2">
+        <v>Person</v>
+      </c>
+      <c r="B1" t="str" s="2">
+        <v>School</v>
+      </c>
+      <c r="C1" t="str" s="2">
+        <v>Degree</v>
+      </c>
+      <c r="D1" t="str" s="2">
+        <v>Field</v>
+      </c>
+      <c r="E1" t="str" s="2">
+        <v>Start</v>
+      </c>
+      <c r="F1" t="str" s="2">
+        <v>End</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str" s="2">
+        <v>Field</v>
+      </c>
+      <c r="B1" t="str" s="2">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B2" t="str" s="3">
+        <v>Alex Rivera</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Photo</v>
+      </c>
+      <c r="B3" t="str" s="3">
+        <v>demo/photos/alex-rivera.jpg</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Role</v>
+      </c>
+      <c r="B4" t="str" s="3">
+        <v>MBA Candidate</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Headline</v>
+      </c>
+      <c r="B5" t="str" s="3">
+        <v>Stanford MBA '27 · Looking for strategy &amp; product roles</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Company</v>
+      </c>
+      <c r="B6" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Schools</v>
+      </c>
+      <c r="B7" t="str" s="3">
+        <v>Stanford University (2025–2027); University of Utah (2016–2020)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Past Companies</v>
+      </c>
+      <c r="B8" t="str" s="3">
+        <v>Delta Air Lines (2020–2022); Adobe (2022–2025)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Email</v>
+      </c>
+      <c r="B9" t="str" s="3">
+        <v>alex.rivera@example.com</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>LinkedIn URL</v>
+      </c>
+      <c r="B10" t="str" s="3">
+        <v>https://www.linkedin.com/in/alex-rivera-demo</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Location</v>
+      </c>
+      <c r="B11" t="str" s="3">
+        <v>Palo Alto, California</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>What I'm looking for</v>
+      </c>
+      <c r="B12" t="str" xml:space="preserve" s="3">
+        <v xml:space="preserve">Summer 2027 internships in strategy or product at consumer-tech and airline companies.
+Happy to swap notes on case prep and product sense interviews.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B9"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str" s="2">
+        <v>Setting</v>
+      </c>
+      <c r="B1" t="str" s="2">
+        <v>Value</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Your name</v>
+      </c>
+      <c r="B2" t="str" s="3">
+        <v>Alex Rivera</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Avatar style</v>
+      </c>
+      <c r="B3" t="str" s="3">
+        <v>notionists</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Your email</v>
+      </c>
+      <c r="B4" t="str" s="3">
+        <v>alex.rivera@example.com</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Meeting length (minutes)</v>
+      </c>
+      <c r="B5" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Zoom link</v>
+      </c>
+      <c r="B6" t="str" s="3">
+        <v>https://zoom.us/j/0000000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Check-in every (days)</v>
+      </c>
+      <c r="B7" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Invite message</v>
+      </c>
+      <c r="B8" t="str" s="3">
+        <v>Hi {first name}, looking forward to our chat on {date} at {time}. {link}</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Demo base date</v>
+      </c>
+      <c r="B9" t="str" s="3">
+        <v>2026-09-28</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C1"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="36.83203125"/>
-    <col min="2" max="2" customWidth="1" width="8.83203125"/>
-    <col min="3" max="3" customWidth="1" width="8.83203125"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1403,12 +2243,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B21"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="110.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="22.83203125"/>
+    <col min="2" max="2" customWidth="1" width="110.83203125"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1586,27 +2426,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D7"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="28.83203125"/>
-    <col min="2" max="2" customWidth="1" width="10.83203125"/>
-    <col min="3" max="3" customWidth="1" width="14.83203125"/>
-    <col min="4" max="4" customWidth="1" width="40.83203125"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="49.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Priority</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Stage</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>Notes</v>
       </c>
     </row>
@@ -1620,7 +2460,7 @@
       <c r="C2" t="str">
         <v>Networking</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" t="str" s="3">
         <v>Strategy practice</v>
       </c>
     </row>
@@ -1634,7 +2474,7 @@
       <c r="C3" t="str">
         <v>Applied</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -1648,7 +2488,7 @@
       <c r="C4" t="str">
         <v>Researching</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4" t="str" s="3">
         <v>Three pool contacts there aren't on the map yet</v>
       </c>
     </row>
@@ -1662,7 +2502,7 @@
       <c r="C5" t="str">
         <v>Researching</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5" t="str" s="3">
         <v>Reachable only through Liam</v>
       </c>
     </row>
@@ -1676,7 +2516,7 @@
       <c r="C6" t="str">
         <v>Researching</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6" t="str" s="3">
         <v>No one yet</v>
       </c>
     </row>
@@ -1690,34 +2530,42 @@
       <c r="C7" t="str">
         <v>Researching</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7" t="str" s="3">
         <v>No one yet</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="B2:B1000">
+      <formula1>"1,2,3"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="C2:C1000">
+      <formula1>"Researching,Networking,Applied,Interviewing,Offer"</formula1>
+    </dataValidation>
+  </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="28.83203125"/>
-    <col min="2" max="2" customWidth="1" width="30.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Website</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Logo</v>
       </c>
     </row>
@@ -1849,39 +2697,39 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G27"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="14.83203125"/>
-    <col min="2" max="2" customWidth="1" width="16.83203125"/>
-    <col min="3" max="3" customWidth="1" width="40.83203125"/>
-    <col min="4" max="4" customWidth="1" width="28.83203125"/>
-    <col min="5" max="5" customWidth="1" width="28.83203125"/>
-    <col min="6" max="6" customWidth="1" width="30.83203125"/>
-    <col min="7" max="7" customWidth="1" width="14.83203125"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>First Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Last Name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>URL</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>Email Address</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" t="str" s="2">
         <v>Position</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" t="str" s="2">
         <v>Connected On</v>
       </c>
     </row>
@@ -2484,61 +3332,90 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G27"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" tooltip="https://www.linkedin.com/in/jordan-lee-3f9a21" display="https://www.linkedin.com/in/jordan-lee-3f9a21"/>
+    <hyperlink ref="C3" r:id="rId2" tooltip="https://www.linkedin.com/in/priya-shah-77b0c4" display="https://www.linkedin.com/in/priya-shah-77b0c4"/>
+    <hyperlink ref="C4" r:id="rId3" tooltip="https://www.linkedin.com/in/sofia-alvarez-5d2e18" display="https://www.linkedin.com/in/sofia-alvarez-5d2e18"/>
+    <hyperlink ref="C5" r:id="rId4" tooltip="https://www.linkedin.com/in/noah-carter-a41b77" display="https://www.linkedin.com/in/noah-carter-a41b77"/>
+    <hyperlink ref="C6" r:id="rId5" tooltip="https://www.linkedin.com/in/mia-chen-0c8e42" display="https://www.linkedin.com/in/mia-chen-0c8e42"/>
+    <hyperlink ref="C7" r:id="rId6" tooltip="https://www.linkedin.com/in/kai-morgan-2b6f90" display="https://www.linkedin.com/in/kai-morgan-2b6f90"/>
+    <hyperlink ref="C8" r:id="rId7" tooltip="https://www.linkedin.com/in/elena-rossi-91cd03" display="https://www.linkedin.com/in/elena-rossi-91cd03"/>
+    <hyperlink ref="C9" r:id="rId8" tooltip="https://www.linkedin.com/in/theo-grant-e7a215" display="https://www.linkedin.com/in/theo-grant-e7a215"/>
+    <hyperlink ref="C10" r:id="rId9" tooltip="https://www.linkedin.com/in/nora-singh-48fa6b" display="https://www.linkedin.com/in/nora-singh-48fa6b"/>
+    <hyperlink ref="C11" r:id="rId10" tooltip="https://www.linkedin.com/in/maya-patel-6a1d3e" display="https://www.linkedin.com/in/maya-patel-6a1d3e"/>
+    <hyperlink ref="C12" r:id="rId11" tooltip="https://www.linkedin.com/in/lucas-bennett-c03f59" display="https://www.linkedin.com/in/lucas-bennett-c03f59"/>
+    <hyperlink ref="C13" r:id="rId12" tooltip="https://www.linkedin.com/in/aisha-rahman-8e47b2" display="https://www.linkedin.com/in/aisha-rahman-8e47b2"/>
+    <hyperlink ref="C14" r:id="rId13" tooltip="https://www.linkedin.com/in/diego-santos-1f9c6d" display="https://www.linkedin.com/in/diego-santos-1f9c6d"/>
+    <hyperlink ref="C15" r:id="rId14" tooltip="https://www.linkedin.com/in/hannah-brooks-5b27a0" display="https://www.linkedin.com/in/hannah-brooks-5b27a0"/>
+    <hyperlink ref="C16" r:id="rId15" tooltip="https://www.linkedin.com/in/omar-haddad-3d81fe" display="https://www.linkedin.com/in/omar-haddad-3d81fe"/>
+    <hyperlink ref="C17" r:id="rId16" tooltip="https://www.linkedin.com/in/grace-liu-9a0e6c" display="https://www.linkedin.com/in/grace-liu-9a0e6c"/>
+    <hyperlink ref="C18" r:id="rId17" tooltip="https://www.linkedin.com/in/ryan-doyle-4c5b12" display="https://www.linkedin.com/in/ryan-doyle-4c5b12"/>
+    <hyperlink ref="C19" r:id="rId18" tooltip="https://www.linkedin.com/in/chloe-martin-b8d4a7" display="https://www.linkedin.com/in/chloe-martin-b8d4a7"/>
+    <hyperlink ref="C20" r:id="rId19" tooltip="https://www.linkedin.com/in/ben-walker-0e3c95" display="https://www.linkedin.com/in/ben-walker-0e3c95"/>
+    <hyperlink ref="C21" r:id="rId20" tooltip="https://www.linkedin.com/in/isabel-cruz-7f2a48" display="https://www.linkedin.com/in/isabel-cruz-7f2a48"/>
+    <hyperlink ref="C22" r:id="rId21" tooltip="https://www.linkedin.com/in/ethan-park-2d6e91" display="https://www.linkedin.com/in/ethan-park-2d6e91"/>
+    <hyperlink ref="C23" r:id="rId22" tooltip="https://www.linkedin.com/in/zara-ahmed-c4b710" display="https://www.linkedin.com/in/zara-ahmed-c4b710"/>
+    <hyperlink ref="C24" r:id="rId23" tooltip="https://www.linkedin.com/in/leo-fischer-6e0d2b" display="https://www.linkedin.com/in/leo-fischer-6e0d2b"/>
+    <hyperlink ref="C25" r:id="rId24" tooltip="https://www.linkedin.com/in/emma-nguyen-93a5f4" display="https://www.linkedin.com/in/emma-nguyen-93a5f4"/>
+    <hyperlink ref="C26" r:id="rId25" tooltip="https://www.linkedin.com/in/jack-sullivan-1b8e07" display="https://www.linkedin.com/in/jack-sullivan-1b8e07"/>
+    <hyperlink ref="C27" r:id="rId26" tooltip="https://www.linkedin.com/in/olivia-reed-58c9d3" display="https://www.linkedin.com/in/olivia-reed-58c9d3"/>
+  </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:G27"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K10"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="22.83203125"/>
-    <col min="2" max="2" customWidth="1" width="12.83203125"/>
-    <col min="3" max="3" customWidth="1" width="8.83203125"/>
-    <col min="4" max="4" customWidth="1" width="8.83203125"/>
-    <col min="5" max="5" customWidth="1" width="16.83203125"/>
-    <col min="6" max="6" customWidth="1" width="12.83203125"/>
-    <col min="7" max="7" customWidth="1" width="40.83203125"/>
-    <col min="8" max="8" customWidth="1" width="30.83203125"/>
-    <col min="9" max="9" customWidth="1" width="22.83203125"/>
-    <col min="10" max="10" customWidth="1" width="30.83203125"/>
-    <col min="11" max="11" customWidth="1" width="16.83203125"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" customWidth="1"/>
+    <col min="10" max="10" width="38.83203125" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Person</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Date</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Start</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>End</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" t="str" s="2">
         <v>Type</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" t="str" s="2">
         <v>Method</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" t="str" s="2">
         <v>Notes</v>
       </c>
-      <c r="H1" t="str">
+      <c r="H1" t="str" s="2">
         <v>Next Step</v>
       </c>
-      <c r="I1" t="str">
+      <c r="I1" t="str" s="2">
         <v>Calendar Event ID</v>
       </c>
-      <c r="J1" t="str">
+      <c r="J1" t="str" s="2">
         <v>Link</v>
       </c>
-      <c r="K1" t="str">
+      <c r="K1" t="str" s="2">
         <v>ID</v>
       </c>
     </row>
@@ -2561,10 +3438,10 @@
       <c r="F2" t="str">
         <v>In Person</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" s="3">
         <v>Caught up; he offered to introduce me to Zoe at Qualtrics.</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H2" t="str" s="3">
         <v>Ask Liam for the Zoe intro</v>
       </c>
       <c r="I2" t="str">
@@ -2596,10 +3473,10 @@
       <c r="F3" t="str">
         <v>In Person</v>
       </c>
-      <c r="G3" t="str">
+      <c r="G3" t="str" s="3">
         <v>Marketplace roadmap, how PMs at Microsoft pick problems.</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H3" t="str" s="3">
         <v>Send thank-you</v>
       </c>
       <c r="I3" t="str">
@@ -2631,10 +3508,10 @@
       <c r="F4" t="str">
         <v>Zoom</v>
       </c>
-      <c r="G4" t="str">
+      <c r="G4" t="str" s="3">
         <v>Walked through case interview prep and the strategy practice.</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H4" t="str" s="3">
         <v>Send resume for review</v>
       </c>
       <c r="I4" t="str">
@@ -2666,10 +3543,10 @@
       <c r="F5" t="str">
         <v>Phone</v>
       </c>
-      <c r="G5" t="str">
+      <c r="G5" t="str" s="3">
         <v>Delta's commercial strategy team; APM-style rotation.</v>
       </c>
-      <c r="H5" t="str">
+      <c r="H5" t="str" s="3">
         <v>Apply to the fall rotation</v>
       </c>
       <c r="I5" t="str">
@@ -2701,10 +3578,10 @@
       <c r="F6" t="str">
         <v>Zoom</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G6" t="str" s="3">
         <v>Goldman strategy group; offered to connect me with Ben.</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H6" t="str" s="3">
         <v>Send thank-you</v>
       </c>
       <c r="I6" t="str">
@@ -2736,10 +3613,10 @@
       <c r="F7" t="str">
         <v>Zoom</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
+      <c r="G7" t="str" s="3">
+        <v/>
+      </c>
+      <c r="H7" t="str" s="3">
         <v/>
       </c>
       <c r="I7" t="str">
@@ -2771,10 +3648,10 @@
       <c r="F8" t="str">
         <v>Teams</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G8" t="str" s="3">
         <v>Recruiter screen for the Delta internship.</v>
       </c>
-      <c r="H8" t="str">
+      <c r="H8" t="str" s="3">
         <v/>
       </c>
       <c r="I8" t="str">
@@ -2806,10 +3683,10 @@
       <c r="F9" t="str">
         <v>Google Meet</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
+      <c r="G9" t="str" s="3">
+        <v/>
+      </c>
+      <c r="H9" t="str" s="3">
         <v/>
       </c>
       <c r="I9" t="str">
@@ -2841,10 +3718,10 @@
       <c r="F10" t="str">
         <v>Zoom</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
+      <c r="G10" t="str" s="3">
+        <v/>
+      </c>
+      <c r="H10" t="str" s="3">
         <v/>
       </c>
       <c r="I10" t="str">
@@ -2858,54 +3735,62 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="E2:E1000">
+      <formula1>"Coffee Chat,Informational,Networking Event,Class/Club,Interview,Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="F2:F1000">
+      <formula1>"Zoom,Google Meet,Teams,Phone,In Person,Email,LinkedIn"</formula1>
+    </dataValidation>
+  </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H10"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="40.83203125"/>
-    <col min="2" max="2" customWidth="1" width="22.83203125"/>
-    <col min="3" max="3" customWidth="1" width="20.83203125"/>
-    <col min="4" max="4" customWidth="1" width="12.83203125"/>
-    <col min="5" max="5" customWidth="1" width="8.83203125"/>
-    <col min="6" max="6" customWidth="1" width="12.83203125"/>
-    <col min="7" max="7" customWidth="1" width="20.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="1" max="1" width="53.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Task</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Person</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>Due</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" t="str" s="2">
         <v>Done</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" t="str" s="2">
         <v>Created</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" t="str" s="2">
         <v>Source</v>
       </c>
-      <c r="H1" t="str">
+      <c r="H1" t="str" s="2">
         <v>ID</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" t="str" s="3">
         <v>Send thank-you to Daniel Ortiz within 24 hrs</v>
       </c>
       <c r="B2" t="str">
@@ -2931,7 +3816,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3" t="str" s="3">
         <v>Follow up with Hana Kim about the strategy practice</v>
       </c>
       <c r="B3" t="str">
@@ -2957,7 +3842,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4" t="str" s="3">
         <v>Send resume to Jordan for review</v>
       </c>
       <c r="B4" t="str">
@@ -2983,7 +3868,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5" t="str" s="3">
         <v>Prepare questions for coffee chat with Priya</v>
       </c>
       <c r="B5" t="str">
@@ -3009,7 +3894,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6" t="str" s="3">
         <v>Ask Liam for the intro to Zoe Adams</v>
       </c>
       <c r="B6" t="str">
@@ -3035,7 +3920,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7" t="str" s="3">
         <v>Research Apple strategy &amp; operations roles</v>
       </c>
       <c r="B7" t="str">
@@ -3061,7 +3946,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8" t="str" s="3">
         <v>Update resume with fall projects</v>
       </c>
       <c r="B8" t="str">
@@ -3087,7 +3972,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9" t="str" s="3">
         <v>Send thank-you to Noah Carter within 24 hrs</v>
       </c>
       <c r="B9" t="str">
@@ -3113,7 +3998,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10" t="str" s="3">
         <v>Send thank-you to Sofia Alvarez within 24 hrs</v>
       </c>
       <c r="B10" t="str">
@@ -3139,33 +4024,38 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="E2:E1000">
+      <formula1>"Yes"</formula1>
+    </dataValidation>
+  </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D13"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="24.83203125"/>
-    <col min="2" max="2" customWidth="1" width="24.83203125"/>
-    <col min="3" max="3" customWidth="1" width="16.83203125"/>
-    <col min="4" max="4" customWidth="1" width="40.83203125"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" t="str" s="2">
         <v>Person A</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" t="str" s="2">
         <v>Person B</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" t="str" s="2">
         <v>Type</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" t="str" s="2">
         <v>Notes</v>
       </c>
     </row>
@@ -3179,7 +4069,7 @@
       <c r="C2" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3193,7 +4083,7 @@
       <c r="C3" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3207,7 +4097,7 @@
       <c r="C4" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3221,7 +4111,7 @@
       <c r="C5" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3235,7 +4125,7 @@
       <c r="C6" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3249,7 +4139,7 @@
       <c r="C7" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3263,7 +4153,7 @@
       <c r="C8" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D8" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3277,7 +4167,7 @@
       <c r="C9" t="str">
         <v>Introduced me</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D9" t="str" s="3">
         <v/>
       </c>
     </row>
@@ -3291,7 +4181,7 @@
       <c r="C10" t="str">
         <v>Friend</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10" t="str" s="3">
         <v>Roommates' friend group</v>
       </c>
     </row>
@@ -3305,7 +4195,7 @@
       <c r="C11" t="str">
         <v>Classmate</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11" t="str" s="3">
         <v>Stanford, same product club</v>
       </c>
     </row>
@@ -3319,7 +4209,7 @@
       <c r="C12" t="str">
         <v>Mentor</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12" t="str" s="3">
         <v>Jordan mentors Owen on case interviews</v>
       </c>
     </row>
@@ -3333,212 +4223,61 @@
       <c r="C13" t="str">
         <v>Coworker</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D13" t="str" s="3">
         <v>Worked together at Deloitte</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" errorStyle="information" sqref="C2:C1000">
+      <formula1>"Introduced me,Coworker,Classmate,Friend,Mentor,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:G1"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="22.83203125"/>
-    <col min="2" max="2" customWidth="1" width="70.83203125"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Name</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Alex Rivera</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Photo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>demo/photos/alex-rivera.jpg</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Role</v>
-      </c>
-      <c r="B4" t="str">
-        <v>MBA Candidate</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Headline</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Stanford MBA '27 · Looking for strategy &amp; product roles</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
+      <c r="A1" t="str" s="2">
+        <v>Person</v>
+      </c>
+      <c r="B1" t="str" s="2">
         <v>Company</v>
       </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Schools</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Stanford University (2025–2027); University of Utah (2016–2020)</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Past Companies</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Delta Air Lines (2020–2022); Adobe (2022–2025)</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Email</v>
-      </c>
-      <c r="B9" t="str">
-        <v>alex.rivera@example.com</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>LinkedIn URL</v>
-      </c>
-      <c r="B10" t="str">
-        <v>https://www.linkedin.com/in/alex-rivera-demo</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
+      <c r="C1" t="str" s="2">
+        <v>Title</v>
+      </c>
+      <c r="D1" t="str" s="2">
+        <v>Start</v>
+      </c>
+      <c r="E1" t="str" s="2">
+        <v>End</v>
+      </c>
+      <c r="F1" t="str" s="2">
         <v>Location</v>
       </c>
-      <c r="B11" t="str">
-        <v>Palo Alto, California</v>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12" t="str">
-        <v>What I'm looking for</v>
-      </c>
-      <c r="B12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Summer 2027 internships in strategy or product at consumer-tech and airline companies.
-Happy to swap notes on case prep and product sense interviews.</v>
+      <c r="G1" t="str" s="2">
+        <v>Description</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
-  <cols>
-    <col min="1" max="1" customWidth="1" width="26.83203125"/>
-    <col min="2" max="2" customWidth="1" width="60.83203125"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Setting</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Your name</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Alex Rivera</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Avatar style</v>
-      </c>
-      <c r="B3" t="str">
-        <v>notionists</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Your email</v>
-      </c>
-      <c r="B4" t="str">
-        <v>alex.rivera@example.com</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Meeting length (minutes)</v>
-      </c>
-      <c r="B5">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Zoom link</v>
-      </c>
-      <c r="B6" t="str">
-        <v>https://zoom.us/j/0000000000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Check-in every (days)</v>
-      </c>
-      <c r="B7">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Invite message</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Hi {first name}, looking forward to our chat on {date} at {time}. {link}</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Demo base date</v>
-      </c>
-      <c r="B9" t="str">
-        <v>2026-09-28</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixes part 7: company and school dots appear on their own
As soon as 3 or more people on the map share a company (current or past,
matched through the name aliases) or a school, that company or school gets its
own node with its logo, live on every add, edit, import and merge. Direct
members hang off it, 2nd-degree members get a secondary link, and past
employees a faint alumni link. Below the threshold the node goes away unless
it's a target. The threshold is a setting (default 3, Settings sheet "Group
size (people)"), and a toast says "Created Adobe group (3 people)".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -2131,7 +2131,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -2203,15 +2203,23 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Group size (people)</v>
+      </c>
+      <c r="B9" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>Demo base date</v>
       </c>
-      <c r="B9" t="str" s="3">
+      <c r="B10" t="str" s="3">
         <v>2026-09-28</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3369,7 +3377,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:Q10"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3382,6 +3390,12 @@
     <col min="9" max="9" width="19.83203125" customWidth="1"/>
     <col min="10" max="10" width="38.83203125" customWidth="1"/>
     <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3418,6 +3432,24 @@
       <c r="K1" t="str" s="2">
         <v>ID</v>
       </c>
+      <c r="L1" t="str" s="2">
+        <v>Title</v>
+      </c>
+      <c r="M1" t="str" s="2">
+        <v>Guests</v>
+      </c>
+      <c r="N1" t="str" s="2">
+        <v>Location</v>
+      </c>
+      <c r="O1" t="str" s="2">
+        <v>Description</v>
+      </c>
+      <c r="P1" t="str" s="2">
+        <v>Reminder (min)</v>
+      </c>
+      <c r="Q1" t="str" s="2">
+        <v>Time Zone</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3453,6 +3485,24 @@
       <c r="K2" t="str">
         <v>demo-m1</v>
       </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -3488,6 +3538,24 @@
       <c r="K3" t="str">
         <v>demo-m2</v>
       </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3523,6 +3591,24 @@
       <c r="K4" t="str">
         <v>demo-m3</v>
       </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3558,6 +3644,24 @@
       <c r="K5" t="str">
         <v>demo-m4</v>
       </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3593,6 +3697,24 @@
       <c r="K6" t="str">
         <v>demo-m5</v>
       </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3628,6 +3750,24 @@
       <c r="K7" t="str">
         <v>demo-m6</v>
       </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -3663,6 +3803,24 @@
       <c r="K8" t="str">
         <v>demo-m7</v>
       </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -3698,6 +3856,24 @@
       <c r="K9" t="str">
         <v>demo-m8</v>
       </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -3732,6 +3908,24 @@
       </c>
       <c r="K10" t="str">
         <v>demo-m9</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str" s="3">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3744,7 +3938,7 @@
     </dataValidation>
   </dataValidations>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phase 7: Pages workflow, demo work history, legacy pdf.js, README GIF
- .github/workflows/pages.yml: tests on Node 22, then deploy site/ to GitHub Pages.
- pdf.js legacy build (same version) so PDF import works in older browsers and Node 22.
- Demo: Sofia, Jordan and Noah get a full work history (timeline in their details).
- The multi-role PDF fixture is now a clearly fictional healthcare career.
- README: live demo link and a GIF tour (docs/orbit-demo.gif) instead of the old screenshot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -443,15 +443,15 @@
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="17.83203125" customWidth="1"/>
     <col min="12" max="12" width="30.83203125" customWidth="1"/>
-    <col min="13" max="13" width="16.83203125" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="29.83203125" customWidth="1"/>
+    <col min="14" max="14" width="53.83203125" customWidth="1"/>
+    <col min="15" max="15" width="27.83203125" customWidth="1"/>
     <col min="16" max="16" width="9.83203125" customWidth="1"/>
-    <col min="17" max="17" width="8.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="52.83203125" customWidth="1"/>
+    <col min="18" max="18" width="31.83203125" customWidth="1"/>
+    <col min="19" max="19" width="31.83203125" customWidth="1"/>
     <col min="20" max="20" width="8.83203125" customWidth="1"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1"/>
+    <col min="21" max="21" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -557,25 +557,25 @@
         <v>Case interview tips</v>
       </c>
       <c r="M2" t="str" s="3">
-        <v/>
+        <v>Delta Air Lines (2019–2019)</v>
       </c>
       <c r="N2" t="str" s="3">
-        <v/>
+        <v>Senior Consultant, Strategy &amp; Analytics at Deloitte</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>San Francisco, California</v>
       </c>
       <c r="P2" t="str">
         <v/>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>Market Sizing; Financial Modeling; Case Interviews</v>
       </c>
       <c r="R2" t="str">
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>Certified Scrum Product Owner</v>
       </c>
       <c r="T2" t="str">
         <v/>
@@ -687,22 +687,22 @@
         <v>Owns the marketplace roadmap</v>
       </c>
       <c r="M4" t="str" s="3">
-        <v/>
+        <v>Deloitte (2018–2021)</v>
       </c>
       <c r="N4" t="str" s="3">
-        <v/>
+        <v>Product Manager at Microsoft · Marketplace</v>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>Seattle, Washington</v>
       </c>
       <c r="P4" t="str">
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v/>
+        <v>Product Strategy; SQL; Experimentation</v>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>Spanish (Native or Bilingual)</v>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -711,7 +711,7 @@
         <v/>
       </c>
       <c r="U4" t="str" s="3">
-        <v/>
+        <v>PM for the Microsoft marketplace. Former Deloitte consultant; Stanford GSB.</v>
       </c>
     </row>
     <row r="5">
@@ -755,16 +755,16 @@
         <v/>
       </c>
       <c r="N5" t="str" s="3">
-        <v/>
+        <v>Commercial Strategy Analyst at Delta Air Lines</v>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>Atlanta, Georgia</v>
       </c>
       <c r="P5" t="str">
         <v/>
       </c>
       <c r="Q5" t="str">
-        <v/>
+        <v>Network Planning; Forecasting; Python</v>
       </c>
       <c r="R5" t="str">
         <v/>
@@ -1980,12 +1980,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="41.83203125" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
   </cols>
@@ -2010,9 +2010,89 @@
         <v>End</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Stanford University</v>
+      </c>
+      <c r="C2" t="str" s="3">
+        <v>Master of Business Administration - MBA</v>
+      </c>
+      <c r="D2" t="str" s="3">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>2021</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B3" t="str">
+        <v>University of Utah</v>
+      </c>
+      <c r="C3" t="str" s="3">
+        <v>Bachelor of Science - BS</v>
+      </c>
+      <c r="D3" t="str" s="3">
+        <v>Information Systems</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2014</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Stanford University</v>
+      </c>
+      <c r="C4" t="str" s="3">
+        <v>Bachelor of Arts - BA</v>
+      </c>
+      <c r="D4" t="str" s="3">
+        <v>Economics</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2016</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Noah Carter</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Stanford University</v>
+      </c>
+      <c r="C5" t="str" s="3">
+        <v>Master of Science - MS</v>
+      </c>
+      <c r="D5" t="str" s="3">
+        <v>Management Science &amp; Engineering</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2019</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2021</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4435,15 +4515,15 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G9"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="41.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" customWidth="1"/>
+    <col min="5" max="5" width="9.83203125" customWidth="1"/>
+    <col min="6" max="6" width="27.83203125" customWidth="1"/>
+    <col min="7" max="7" width="49.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4469,9 +4549,193 @@
         <v>Description</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Microsoft</v>
+      </c>
+      <c r="C2" t="str" s="3">
+        <v>Product Manager</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2023-07</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Present</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Redmond, Washington</v>
+      </c>
+      <c r="G2" t="str" s="3">
+        <v>Owns the marketplace roadmap and pricing tests.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Microsoft</v>
+      </c>
+      <c r="C3" t="str" s="3">
+        <v>Product Manager Intern</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2022-06</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2022-09</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Redmond, Washington</v>
+      </c>
+      <c r="G3" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Sofia Alvarez</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Deloitte</v>
+      </c>
+      <c r="C4" t="str" s="3">
+        <v>Business Technology Analyst</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2018-08</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2021-06</v>
+      </c>
+      <c r="F4" t="str">
+        <v>San Francisco Bay Area</v>
+      </c>
+      <c r="G4" t="str" s="3">
+        <v>Tech strategy for retail and travel clients.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Deloitte</v>
+      </c>
+      <c r="C5" t="str" s="3">
+        <v>Strategy &amp; Analytics: Senior Consultant</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2022-01</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Present</v>
+      </c>
+      <c r="F5" t="str">
+        <v>San Francisco, California</v>
+      </c>
+      <c r="G5" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Deloitte</v>
+      </c>
+      <c r="C6" t="str" s="3">
+        <v>Strategy &amp; Analytics: Consultant</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2020-08</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2021-12</v>
+      </c>
+      <c r="F6" t="str">
+        <v>San Francisco, California</v>
+      </c>
+      <c r="G6" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Jordan Lee</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Delta Air Lines</v>
+      </c>
+      <c r="C7" t="str" s="3">
+        <v>Revenue Management Intern</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2019-06</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2019-08</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Atlanta, Georgia</v>
+      </c>
+      <c r="G7" t="str" s="3">
+        <v>Pricing analysis for transatlantic routes.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Noah Carter</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Delta Air Lines</v>
+      </c>
+      <c r="C8" t="str" s="3">
+        <v>Commercial Strategy Analyst</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2023-02</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Present</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Atlanta, Georgia</v>
+      </c>
+      <c r="G8" t="str" s="3">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Noah Carter</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Delta Air Lines</v>
+      </c>
+      <c r="C9" t="str" s="3">
+        <v>Network Planning Analyst</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2021-07</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2023-01</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Atlanta, Georgia</v>
+      </c>
+      <c r="G9" t="str" s="3">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Round 2, group B: a simpler demo; edit any school or company dot
- The demo keeps all 22 people but only four organizations: Stanford University
  (school), Microsoft and Deloitte (company groups) and Google (a target with no
  one yet). Past companies stay in work histories but stay under the group size.
- Every company / school dot has an Edit button: type (School or Company; changing
  it moves the value between people's Schools and Company / Past Companies),
  website, and picture (upload, image link, or find automatically), saved in the
  Companies sheet.
- Tests updated for the new demo; a new test covers changing a dot's type.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -434,7 +434,7 @@
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="21.83203125" customWidth="1"/>
     <col min="3" max="3" width="21.83203125" customWidth="1"/>
-    <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="4" max="4" width="27.83203125" customWidth="1"/>
     <col min="5" max="5" width="27.83203125" customWidth="1"/>
     <col min="6" max="6" width="50.83203125" customWidth="1"/>
     <col min="7" max="7" width="31.83203125" customWidth="1"/>
@@ -557,7 +557,7 @@
         <v>Case interview tips</v>
       </c>
       <c r="M2" t="str" s="3">
-        <v>Delta Air Lines (2019–2019)</v>
+        <v>Adobe (2019–2019)</v>
       </c>
       <c r="N2" t="str" s="3">
         <v>Senior Consultant, Strategy &amp; Analytics at Deloitte</v>
@@ -592,7 +592,7 @@
         <v>Deloitte</v>
       </c>
       <c r="C3" t="str" s="3">
-        <v>University of Utah</v>
+        <v>Stanford University</v>
       </c>
       <c r="D3" t="str">
         <v>Manager</v>
@@ -719,13 +719,13 @@
         <v>Noah Carter</v>
       </c>
       <c r="B5" t="str">
-        <v>Delta Air Lines</v>
+        <v>Microsoft</v>
       </c>
       <c r="C5" t="str" s="3">
         <v>Stanford University</v>
       </c>
       <c r="D5" t="str">
-        <v>Commercial Strategy Analyst</v>
+        <v>Business Strategy Analyst</v>
       </c>
       <c r="E5" t="str">
         <v>noah.carter@example.com</v>
@@ -752,19 +752,19 @@
         <v>Info session speaker</v>
       </c>
       <c r="M5" t="str" s="3">
-        <v/>
+        <v>Delta Air Lines (2021–2023)</v>
       </c>
       <c r="N5" t="str" s="3">
-        <v>Commercial Strategy Analyst at Delta Air Lines</v>
+        <v>Business Strategy Analyst at Microsoft</v>
       </c>
       <c r="O5" t="str">
-        <v>Atlanta, Georgia</v>
+        <v>Seattle, Washington</v>
       </c>
       <c r="P5" t="str">
         <v/>
       </c>
       <c r="Q5" t="str">
-        <v>Network Planning; Forecasting; Python</v>
+        <v>Forecasting; Customer Research; Python</v>
       </c>
       <c r="R5" t="str">
         <v/>
@@ -784,10 +784,10 @@
         <v>Mia Chen</v>
       </c>
       <c r="B6" t="str">
-        <v>Google</v>
+        <v>Microsoft</v>
       </c>
       <c r="C6" t="str" s="3">
-        <v>University of Utah</v>
+        <v>Stanford University</v>
       </c>
       <c r="D6" t="str">
         <v>Product Lead</v>
@@ -1047,7 +1047,7 @@
         <v>Microsoft</v>
       </c>
       <c r="C10" t="str" s="3">
-        <v>University of Utah</v>
+        <v/>
       </c>
       <c r="D10" t="str">
         <v>Program Manager</v>
@@ -1109,13 +1109,13 @@
         <v>Grace Owens</v>
       </c>
       <c r="B11" t="str">
-        <v>Delta Air Lines</v>
+        <v>Deloitte</v>
       </c>
       <c r="C11" t="str" s="3">
         <v/>
       </c>
       <c r="D11" t="str">
-        <v>Recruiter</v>
+        <v>Campus Recruiter</v>
       </c>
       <c r="E11" t="str">
         <v>grace.owens@example.com</v>
@@ -1174,7 +1174,7 @@
         <v>Daniel Ortiz</v>
       </c>
       <c r="B12" t="str">
-        <v>Goldman Sachs</v>
+        <v>Deloitte</v>
       </c>
       <c r="C12" t="str" s="3">
         <v>Stanford University</v>
@@ -1239,10 +1239,10 @@
         <v>Owen Price</v>
       </c>
       <c r="B13" t="str">
-        <v>Google</v>
+        <v>Microsoft</v>
       </c>
       <c r="C13" t="str" s="3">
-        <v>University of Utah</v>
+        <v/>
       </c>
       <c r="D13" t="str">
         <v>Associate Product Manager</v>
@@ -1304,10 +1304,10 @@
         <v>Ava Thompson</v>
       </c>
       <c r="B14" t="str">
-        <v>Adobe</v>
+        <v>Microsoft</v>
       </c>
       <c r="C14" t="str" s="3">
-        <v>University of Utah</v>
+        <v/>
       </c>
       <c r="D14" t="str">
         <v>Operations Lead</v>
@@ -1629,13 +1629,13 @@
         <v>Victor Hale</v>
       </c>
       <c r="B19" t="str">
-        <v>Delta Air Lines</v>
+        <v>Microsoft</v>
       </c>
       <c r="C19" t="str" s="3">
         <v/>
       </c>
       <c r="D19" t="str">
-        <v>VP Network Planning</v>
+        <v>VP of Strategy</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -1694,7 +1694,7 @@
         <v>Chloe Park</v>
       </c>
       <c r="B20" t="str">
-        <v>Adobe</v>
+        <v>Microsoft</v>
       </c>
       <c r="C20" t="str" s="3">
         <v/>
@@ -1824,7 +1824,7 @@
         <v>Zoe Adams</v>
       </c>
       <c r="B22" t="str">
-        <v>Qualtrics</v>
+        <v>Microsoft</v>
       </c>
       <c r="C22" t="str" s="3">
         <v/>
@@ -1889,7 +1889,7 @@
         <v>Sam Rivera</v>
       </c>
       <c r="B23" t="str">
-        <v>Qualtrics</v>
+        <v>Microsoft</v>
       </c>
       <c r="C23" t="str" s="3">
         <v/>
@@ -1983,7 +1983,7 @@
   <dimension ref="A1:F5"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="41.83203125" customWidth="1"/>
     <col min="4" max="4" width="34.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
@@ -2035,7 +2035,7 @@
         <v>Sofia Alvarez</v>
       </c>
       <c r="B3" t="str">
-        <v>University of Utah</v>
+        <v>University of Washington</v>
       </c>
       <c r="C3" t="str" s="3">
         <v>Bachelor of Science - BS</v>
@@ -2158,7 +2158,7 @@
         <v>Schools</v>
       </c>
       <c r="B7" t="str" s="3">
-        <v>Stanford University (2025–2027); University of Utah (2016–2020)</v>
+        <v>Stanford University (2025–2027); University of Washington (2016–2020)</v>
       </c>
     </row>
     <row r="8">
@@ -2516,12 +2516,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D4"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="49.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2554,72 +2554,30 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Delta Air Lines</v>
+        <v>Google</v>
       </c>
       <c r="B3" t="str">
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>Applied</v>
+        <v>Researching</v>
       </c>
       <c r="D3" t="str" s="3">
-        <v/>
+        <v>No one on the map yet: two people there are in your LinkedIn pool</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Goldman Sachs</v>
+        <v>Microsoft</v>
       </c>
       <c r="B4" t="str">
         <v>2</v>
       </c>
       <c r="C4" t="str">
-        <v>Researching</v>
+        <v>Networking</v>
       </c>
       <c r="D4" t="str" s="3">
-        <v>Three pool contacts there aren't on the map yet</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Qualtrics</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Researching</v>
-      </c>
-      <c r="D5" t="str" s="3">
-        <v>Reachable only through Liam</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Apple</v>
-      </c>
-      <c r="B6" t="str">
-        <v>3</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Researching</v>
-      </c>
-      <c r="D6" t="str" s="3">
-        <v>No one yet</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Nike</v>
-      </c>
-      <c r="B7" t="str">
-        <v>3</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Researching</v>
-      </c>
-      <c r="D7" t="str" s="3">
-        <v>No one yet</v>
+        <v>Product roles; Sofia is the warmest way in</v>
       </c>
     </row>
   </sheetData>
@@ -2632,7 +2590,7 @@
     </dataValidation>
   </dataValidations>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3551,7 +3509,7 @@
         <v>In Person</v>
       </c>
       <c r="G2" t="str" s="3">
-        <v>Caught up; he offered to introduce me to Zoe at Qualtrics.</v>
+        <v>Caught up; he offered to introduce me to Zoe on Microsoft's strategy team.</v>
       </c>
       <c r="H2" t="str" s="3">
         <v>Ask Liam for the Zoe intro</v>
@@ -3710,7 +3668,7 @@
         <v>Phone</v>
       </c>
       <c r="G5" t="str" s="3">
-        <v>Delta's commercial strategy team; APM-style rotation.</v>
+        <v>Microsoft's business strategy team; APM-style rotation.</v>
       </c>
       <c r="H5" t="str" s="3">
         <v>Apply to the fall rotation</v>
@@ -3763,7 +3721,7 @@
         <v>Zoom</v>
       </c>
       <c r="G6" t="str" s="3">
-        <v>Goldman strategy group; offered to connect me with Ben.</v>
+        <v>Deloitte strategy group; offered to connect me with Ben.</v>
       </c>
       <c r="H6" t="str" s="3">
         <v>Send thank-you</v>
@@ -3869,7 +3827,7 @@
         <v>Teams</v>
       </c>
       <c r="G8" t="str" s="3">
-        <v>Recruiter screen for the Delta internship.</v>
+        <v>Recruiter screen for the Deloitte internship.</v>
       </c>
       <c r="H8" t="str" s="3">
         <v/>
@@ -4029,7 +3987,7 @@
   <cols>
     <col min="1" max="1" width="53.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
@@ -4071,7 +4029,7 @@
         <v>Daniel Ortiz</v>
       </c>
       <c r="C2" t="str">
-        <v>Goldman Sachs</v>
+        <v>Deloitte</v>
       </c>
       <c r="D2" s="1">
         <v>46292</v>
@@ -4175,7 +4133,7 @@
         <v>Liam Walsh</v>
       </c>
       <c r="C6" t="str">
-        <v>Qualtrics</v>
+        <v>Microsoft</v>
       </c>
       <c r="D6" s="1">
         <v>46296</v>
@@ -4195,13 +4153,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str" s="3">
-        <v>Research Apple strategy &amp; operations roles</v>
+        <v>Research Google strategy &amp; operations roles</v>
       </c>
       <c r="B7" t="str">
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>Apple</v>
+        <v>Google</v>
       </c>
       <c r="D7" s="1">
         <v>46302</v>
@@ -4253,7 +4211,7 @@
         <v>Noah Carter</v>
       </c>
       <c r="C9" t="str">
-        <v>Delta Air Lines</v>
+        <v>Microsoft</v>
       </c>
       <c r="D9" s="1">
         <v>46289</v>
@@ -4669,10 +4627,10 @@
         <v>Jordan Lee</v>
       </c>
       <c r="B7" t="str">
-        <v>Delta Air Lines</v>
+        <v>Adobe</v>
       </c>
       <c r="C7" t="str" s="3">
-        <v>Revenue Management Intern</v>
+        <v>Business Strategy Intern</v>
       </c>
       <c r="D7" t="str">
         <v>2019-06</v>
@@ -4681,10 +4639,10 @@
         <v>2019-08</v>
       </c>
       <c r="F7" t="str">
-        <v>Atlanta, Georgia</v>
+        <v>San Jose, California</v>
       </c>
       <c r="G7" t="str" s="3">
-        <v>Pricing analysis for transatlantic routes.</v>
+        <v>Market sizing for a new creative-tools bundle.</v>
       </c>
     </row>
     <row r="8">
@@ -4692,10 +4650,10 @@
         <v>Noah Carter</v>
       </c>
       <c r="B8" t="str">
-        <v>Delta Air Lines</v>
+        <v>Microsoft</v>
       </c>
       <c r="C8" t="str" s="3">
-        <v>Commercial Strategy Analyst</v>
+        <v>Business Strategy Analyst</v>
       </c>
       <c r="D8" t="str">
         <v>2023-02</v>
@@ -4704,7 +4662,7 @@
         <v>Present</v>
       </c>
       <c r="F8" t="str">
-        <v>Atlanta, Georgia</v>
+        <v>Redmond, Washington</v>
       </c>
       <c r="G8" t="str" s="3">
         <v/>
@@ -4718,7 +4676,7 @@
         <v>Delta Air Lines</v>
       </c>
       <c r="C9" t="str" s="3">
-        <v>Network Planning Analyst</v>
+        <v>Loyalty Program Analyst</v>
       </c>
       <c r="D9" t="str">
         <v>2021-07</v>
@@ -4727,7 +4685,7 @@
         <v>2023-01</v>
       </c>
       <c r="F9" t="str">
-        <v>Atlanta, Georgia</v>
+        <v>Seattle, Washington</v>
       </c>
       <c r="G9" t="str" s="3">
         <v/>

</xml_diff>

<commit_message>
Round 2, group C: map behavior
- "No one yet" targets can be dragged like any dot; dragged dots keep their spot.
- The Lock button and feature are gone; Re-arrange stays.
- Legend & view: a "Groups form at: 2-10 people" slider (live preview, saved in
  Settings) and Group by: Company, School, Skills, Languages, Certifications,
  Tags (several at once; languages ignore the proficiency).
- Group counts come from the lines actually drawn: the (N) on a dot, the card and
  "People in this group" all count the same people (current, 2nd-degree,
  alumni). Tested against the edges.
- Search matches any field (name, company, school, role, skills, languages,
  certifications, tags, notes…) and lists matches with the field that matched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -2211,7 +2211,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -2291,15 +2291,23 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Group by</v>
+      </c>
+      <c r="B10" t="str" s="3">
+        <v>company, school</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Demo base date</v>
       </c>
-      <c r="B10" t="str" s="3">
+      <c r="B11" t="str" s="3">
         <v>2026-09-28</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Round 2, group E: calendar and tasks
- Deleting a meeting removes its automatic tasks that aren't done (linked by
  meeting ID: "thanks:<id>", "prep:<id>"); if you edited any of them, it asks
  "Also remove N related tasks?" first. The demo's tasks are linked to their
  meetings. Tested.
- To-Do: the "This week" group no longer picks up the calendar's .week panel
  (the classes are now todo-<group>); a test guards against the clash. Checked
  at narrow and wide widths in both themes.
- The To-Do and LinkedIn Pool footers show just the Orbit mark in the theme color.
- View tabs stay on one line in narrow windows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/demo/demo_network.xlsx
+++ b/site/demo/demo_network.xlsx
@@ -3999,7 +3999,7 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
     <col min="8" max="8" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4049,7 +4049,7 @@
         <v>46289</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>thanks:demo-m5</v>
       </c>
       <c r="H2" t="str">
         <v>demo-t1</v>
@@ -4127,7 +4127,7 @@
         <v>46290</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>prep:demo-m6</v>
       </c>
       <c r="H5" t="str">
         <v>demo-t4</v>
@@ -4231,7 +4231,7 @@
         <v>46286</v>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>thanks:demo-m4</v>
       </c>
       <c r="H9" t="str">
         <v>demo-t8</v>
@@ -4257,7 +4257,7 @@
         <v>46271</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>thanks:demo-m2</v>
       </c>
       <c r="H10" t="str">
         <v>demo-t9</v>

</xml_diff>